<commit_message>
feat(catering-es-2.0): F2 cerrada — los 11 entregables 2.2 en dl/ y gates D12 en verde
- plan financiero (motor de línea A, molde A-β) y checklist (82 tareas) desde el dry-run TODO VERDE
- plan de negocio docx (131 ranuras, 10 H1, A4, 7.426 palabras, 0 tokens sin resolver) y calculadora
  (autotest pycel 168/168)
- D9: 23 arreglos de texto en los otros 7 ficheros (freelance, «validado España 2026», research,
  inversión, RGSEAA, IVA de servicios asociados, estado de proveedores)
- docx p43 (plantilla 3 fijos + 8 fijos discontinuos = {PLANTILLA_PERSONAS}) y p48 (mezcla redondeada
  con prudencia, IVA incluido); gate de cifras prohibidas afinado (2.200 € de seguros es legítimo)
- regresión 5 planes de línea A = 0 diferencias · censo 0 · no latinos 0 · barrido prohibidos 0
- F2-NOTAS.md §6: cierre de la F2

Via: Claude Code

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KriAdpMP6uaswtiVvqtBvP
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/plan-catering-tematico-eventos/plantilla-proveedores-catering-tematico-eventos.xlsx
+++ b/astro-site/public/dl/plan-catering-tematico-eventos/plantilla-proveedores-catering-tematico-eventos.xlsx
@@ -492,11 +492,10 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Validados España 2026 · 12 bloques (cocinas del mundo + equipamiento + servicios)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>12 bloques (cocinas del mundo + equipamiento + servicios) · comprueba disponibilidad y condiciones antes de pedir</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -565,7 +564,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -600,7 +599,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -635,7 +634,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -670,7 +669,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -705,7 +704,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -740,7 +739,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -775,7 +774,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -810,7 +809,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -845,7 +844,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -880,7 +879,7 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -915,7 +914,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -950,7 +949,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -985,7 +984,7 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1019,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1089,7 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1125,7 +1124,7 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1159,7 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1194,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1229,7 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1264,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1299,7 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1334,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1369,7 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1404,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1439,7 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1474,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1545,7 +1544,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1614,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1649,7 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1684,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1754,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1789,7 @@
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1860,7 +1859,7 @@
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1895,7 +1894,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1929,7 @@
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -1965,7 +1964,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2000,7 +1999,7 @@
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2034,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2070,7 +2069,7 @@
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2104,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2139,7 @@
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2174,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2210,7 +2209,7 @@
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2245,7 +2244,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2280,7 +2279,7 @@
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2315,7 +2314,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2349,7 @@
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2385,7 +2384,7 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2420,7 +2419,7 @@
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2455,7 +2454,7 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2489,7 @@
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2525,7 +2524,7 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2560,7 +2559,7 @@
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2594,7 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2630,7 +2629,7 @@
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2665,7 +2664,7 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2700,7 +2699,7 @@
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2734,7 @@
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2770,7 +2769,7 @@
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2804,7 @@
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2840,7 +2839,7 @@
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2874,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2910,7 +2909,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2944,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -2980,7 +2979,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3015,7 +3014,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3050,7 +3049,7 @@
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3085,7 +3084,7 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3120,7 +3119,7 @@
       </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3155,7 +3154,7 @@
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3190,7 +3189,7 @@
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3225,7 +3224,7 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3260,7 +3259,7 @@
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3294,7 @@
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3330,7 +3329,7 @@
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3365,7 +3364,7 @@
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3400,7 +3399,7 @@
       </c>
       <c r="G86" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3434,7 @@
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3469,7 @@
       </c>
       <c r="G88" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3505,7 +3504,7 @@
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3540,7 +3539,7 @@
       </c>
       <c r="G90" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3574,7 @@
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3610,7 +3609,7 @@
       </c>
       <c r="G92" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3644,7 @@
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3680,7 +3679,7 @@
       </c>
       <c r="G94" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3715,7 +3714,7 @@
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3750,7 +3749,7 @@
       </c>
       <c r="G96" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3785,7 +3784,7 @@
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3820,7 +3819,7 @@
       </c>
       <c r="G98" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3855,7 +3854,7 @@
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
@@ -3890,14 +3889,14 @@
       </c>
       <c r="G100" s="5" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Por verificar</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>